<commit_message>
Drive times (no traffic)
</commit_message>
<xml_diff>
--- a/MemberTemplate.xlsx
+++ b/MemberTemplate.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ASCC\Desktop\driverclusters\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A6CFD11-2A28-430F-B49A-CC3FB94331BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{682F8E12-1A31-4841-8A86-3639F5276138}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="780" yWindow="780" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="10980" yWindow="390" windowWidth="17820" windowHeight="15090" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Setup" sheetId="3" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="72">
   <si>
     <t>ID</t>
   </si>
@@ -238,6 +238,15 @@
   </si>
   <si>
     <t>1072 80th St</t>
+  </si>
+  <si>
+    <t>Staten Island</t>
+  </si>
+  <si>
+    <t>118 Cortelyou Ave</t>
+  </si>
+  <si>
+    <t>Shamrock Holmie</t>
   </si>
 </sst>
 </file>
@@ -365,7 +374,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyProtection="1">
@@ -384,10 +393,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyProtection="1">
       <alignment horizontal="right"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyProtection="1">
@@ -698,54 +703,54 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="16" t="s">
         <v>60</v>
       </c>
-      <c r="B1" s="18"/>
+      <c r="B1" s="17"/>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="11" t="s">
+      <c r="A2" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="12" t="s">
+      <c r="B2" s="11" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="11" t="s">
+      <c r="A3" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="12" t="s">
+      <c r="B3" s="11" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="11" t="s">
+      <c r="A4" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="B4" s="12">
+      <c r="B4" s="11">
         <v>11228</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="13">
+      <c r="A5" s="12">
         <v>40.6201972</v>
       </c>
-      <c r="B5" s="14">
+      <c r="B5" s="13">
         <v>-74.015425500000006</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A7" s="17" t="s">
+      <c r="A7" s="16" t="s">
         <v>62</v>
       </c>
-      <c r="B7" s="18"/>
+      <c r="B7" s="17"/>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" s="15" t="s">
+      <c r="A8" s="14" t="s">
         <v>63</v>
       </c>
-      <c r="B8" s="16" t="s">
+      <c r="B8" s="15" t="s">
         <v>64</v>
       </c>
     </row>
@@ -820,33 +825,33 @@
       <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="10" t="s">
+      <c r="H1" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="10" t="s">
+      <c r="I1" s="9" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2" s="8">
+      <c r="A2" s="7">
         <v>1</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="B2" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="C2" s="9">
+      <c r="C2" s="8">
         <v>26658</v>
       </c>
-      <c r="D2" s="8" t="s">
+      <c r="D2" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="E2" s="8" t="s">
+      <c r="E2" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="F2" s="8" t="s">
+      <c r="F2" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="G2" s="8">
+      <c r="G2" s="7">
         <v>11219</v>
       </c>
       <c r="H2">
@@ -857,25 +862,25 @@
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A3" s="8">
+      <c r="A3" s="7">
         <v>2</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="B3" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="9">
+      <c r="C3" s="8">
         <v>23196</v>
       </c>
-      <c r="D3" s="8" t="s">
+      <c r="D3" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="E3" s="8" t="s">
+      <c r="E3" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="F3" s="8" t="s">
+      <c r="F3" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="G3" s="8">
+      <c r="G3" s="7">
         <v>11223</v>
       </c>
       <c r="H3">
@@ -886,25 +891,25 @@
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4" s="8">
+      <c r="A4" s="7">
         <v>3</v>
       </c>
-      <c r="B4" s="8" t="s">
+      <c r="B4" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="C4" s="9">
+      <c r="C4" s="8">
         <v>20028</v>
       </c>
-      <c r="D4" s="8" t="s">
+      <c r="D4" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="E4" s="8" t="s">
+      <c r="E4" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="F4" s="8" t="s">
+      <c r="F4" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="G4" s="8">
+      <c r="G4" s="7">
         <v>11232</v>
       </c>
       <c r="H4">
@@ -915,25 +920,25 @@
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A5" s="8">
+      <c r="A5" s="7">
         <v>4</v>
       </c>
-      <c r="B5" s="8" t="s">
+      <c r="B5" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="C5" s="9">
+      <c r="C5" s="8">
         <v>29384</v>
       </c>
-      <c r="D5" s="8" t="s">
+      <c r="D5" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="E5" s="8" t="s">
+      <c r="E5" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="F5" s="8" t="s">
+      <c r="F5" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="G5" s="8">
+      <c r="G5" s="7">
         <v>11220</v>
       </c>
       <c r="H5">
@@ -944,25 +949,25 @@
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A6" s="8">
+      <c r="A6" s="7">
         <v>5</v>
       </c>
-      <c r="B6" s="8" t="s">
+      <c r="B6" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="C6" s="9">
+      <c r="C6" s="8">
         <v>27474</v>
       </c>
-      <c r="D6" s="8" t="s">
+      <c r="D6" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="E6" s="8" t="s">
+      <c r="E6" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="F6" s="8" t="s">
+      <c r="F6" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="G6" s="8">
+      <c r="G6" s="7">
         <v>11225</v>
       </c>
       <c r="H6">
@@ -973,25 +978,25 @@
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A7" s="8">
+      <c r="A7" s="7">
         <v>6</v>
       </c>
-      <c r="B7" s="8" t="s">
+      <c r="B7" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="C7" s="9">
+      <c r="C7" s="8">
         <v>33191</v>
       </c>
-      <c r="D7" s="8" t="s">
+      <c r="D7" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="E7" s="8" t="s">
+      <c r="E7" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="F7" s="8" t="s">
+      <c r="F7" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="G7" s="8">
+      <c r="G7" s="7">
         <v>11216</v>
       </c>
       <c r="H7">
@@ -1002,25 +1007,25 @@
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A8" s="8">
+      <c r="A8" s="7">
         <v>7</v>
       </c>
-      <c r="B8" s="8" t="s">
+      <c r="B8" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="C8" s="9">
+      <c r="C8" s="8">
         <v>31146</v>
       </c>
-      <c r="D8" s="8" t="s">
+      <c r="D8" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="E8" s="8" t="s">
+      <c r="E8" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="F8" s="8" t="s">
+      <c r="F8" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="G8" s="8">
+      <c r="G8" s="7">
         <v>11203</v>
       </c>
       <c r="H8">
@@ -1031,25 +1036,25 @@
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A9" s="8">
+      <c r="A9" s="7">
         <v>8</v>
       </c>
-      <c r="B9" s="8" t="s">
+      <c r="B9" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="C9" s="9">
+      <c r="C9" s="8">
         <v>34961</v>
       </c>
-      <c r="D9" s="8" t="s">
+      <c r="D9" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="E9" s="8" t="s">
+      <c r="E9" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="F9" s="8" t="s">
+      <c r="F9" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="G9" s="8">
+      <c r="G9" s="7">
         <v>11236</v>
       </c>
       <c r="H9">
@@ -1060,25 +1065,25 @@
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A10" s="8">
+      <c r="A10" s="7">
         <v>9</v>
       </c>
-      <c r="B10" s="8" t="s">
+      <c r="B10" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="C10" s="9">
+      <c r="C10" s="8">
         <v>26328</v>
       </c>
-      <c r="D10" s="8" t="s">
+      <c r="D10" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="E10" s="8" t="s">
+      <c r="E10" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="F10" s="8" t="s">
+      <c r="F10" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="G10" s="8">
+      <c r="G10" s="7">
         <v>11234</v>
       </c>
       <c r="H10">
@@ -1089,25 +1094,25 @@
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A11" s="8">
+      <c r="A11" s="7">
         <v>10</v>
       </c>
-      <c r="B11" s="8" t="s">
+      <c r="B11" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="C11" s="9">
+      <c r="C11" s="8">
         <v>32360</v>
       </c>
-      <c r="D11" s="8" t="s">
+      <c r="D11" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="E11" s="8" t="s">
+      <c r="E11" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="F11" s="8" t="s">
+      <c r="F11" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="G11" s="8">
+      <c r="G11" s="7">
         <v>11208</v>
       </c>
       <c r="H11">
@@ -1118,25 +1123,25 @@
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A12" s="8">
+      <c r="A12" s="7">
         <v>11</v>
       </c>
-      <c r="B12" s="8" t="s">
+      <c r="B12" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="C12" s="9">
+      <c r="C12" s="8">
         <v>25184</v>
       </c>
-      <c r="D12" s="8" t="s">
+      <c r="D12" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="E12" s="8" t="s">
+      <c r="E12" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="F12" s="8" t="s">
+      <c r="F12" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="G12" s="8">
+      <c r="G12" s="7">
         <v>10012</v>
       </c>
       <c r="H12">
@@ -1147,25 +1152,25 @@
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A13" s="8">
+      <c r="A13" s="7">
         <v>12</v>
       </c>
-      <c r="B13" s="8" t="s">
+      <c r="B13" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="C13" s="9">
+      <c r="C13" s="8">
         <v>33749</v>
       </c>
-      <c r="D13" s="8" t="s">
+      <c r="D13" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="E13" s="8" t="s">
+      <c r="E13" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="F13" s="8" t="s">
+      <c r="F13" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="G13" s="8">
+      <c r="G13" s="7">
         <v>10014</v>
       </c>
       <c r="H13">
@@ -1176,25 +1181,25 @@
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A14" s="8">
+      <c r="A14" s="7">
         <v>13</v>
       </c>
-      <c r="B14" s="8" t="s">
+      <c r="B14" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="C14" s="9">
+      <c r="C14" s="8">
         <v>30975</v>
       </c>
-      <c r="D14" s="8" t="s">
+      <c r="D14" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="E14" s="8" t="s">
+      <c r="E14" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="F14" s="8" t="s">
+      <c r="F14" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="G14" s="8">
+      <c r="G14" s="7">
         <v>10007</v>
       </c>
       <c r="H14">
@@ -1205,25 +1210,25 @@
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A15" s="8">
+      <c r="A15" s="7">
         <v>14</v>
       </c>
-      <c r="B15" s="8" t="s">
+      <c r="B15" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="C15" s="9">
+      <c r="C15" s="8">
         <v>29315</v>
       </c>
-      <c r="D15" s="8" t="s">
+      <c r="D15" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="E15" s="8" t="s">
+      <c r="E15" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="F15" s="8" t="s">
+      <c r="F15" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="G15" s="8">
+      <c r="G15" s="7">
         <v>10002</v>
       </c>
       <c r="H15">
@@ -1234,25 +1239,25 @@
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A16" s="8">
+      <c r="A16" s="7">
         <v>15</v>
       </c>
-      <c r="B16" s="8" t="s">
+      <c r="B16" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="C16" s="9">
+      <c r="C16" s="8">
         <v>33065</v>
       </c>
-      <c r="D16" s="8" t="s">
+      <c r="D16" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="E16" s="8" t="s">
+      <c r="E16" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="F16" s="8" t="s">
+      <c r="F16" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="G16" s="8">
+      <c r="G16" s="7">
         <v>10002</v>
       </c>
       <c r="H16">
@@ -1262,14 +1267,34 @@
         <v>-73.982560899999996</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A17" s="7"/>
-      <c r="B17" s="7"/>
-      <c r="C17" s="7"/>
-      <c r="D17" s="7"/>
-      <c r="E17" s="7"/>
-      <c r="F17" s="7"/>
-      <c r="G17" s="7"/>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A17" s="3">
+        <v>16</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="C17" s="8">
+        <v>32562</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="F17" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="G17" s="3">
+        <v>10312</v>
+      </c>
+      <c r="H17">
+        <v>40.55686</v>
+      </c>
+      <c r="I17">
+        <v>-74.164468200000002</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:I16" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
@@ -1316,10 +1341,10 @@
       <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="10" t="s">
+      <c r="H1" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="10" t="s">
+      <c r="I1" s="9" t="s">
         <v>8</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Export to excel setup
</commit_message>
<xml_diff>
--- a/MemberTemplate.xlsx
+++ b/MemberTemplate.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ASCC\Desktop\driverclusters\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{682F8E12-1A31-4841-8A86-3639F5276138}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4090BEAB-39CD-4B06-94C0-EC4E6670AF9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10980" yWindow="390" windowWidth="17820" windowHeight="15090" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="10980" yWindow="390" windowWidth="17820" windowHeight="15090" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Setup" sheetId="3" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="75">
   <si>
     <t>ID</t>
   </si>
@@ -247,6 +247,15 @@
   </si>
   <si>
     <t>Shamrock Holmie</t>
+  </si>
+  <si>
+    <t>Car #</t>
+  </si>
+  <si>
+    <t>ABC1234</t>
+  </si>
+  <si>
+    <t>NYC4567</t>
   </si>
 </sst>
 </file>
@@ -300,7 +309,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -370,11 +379,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyProtection="1">
@@ -416,6 +440,10 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -696,19 +724,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9DF27723-B52E-4D71-B27A-CC03CEF15191}">
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="15.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A1" s="16" t="s">
         <v>60</v>
       </c>
       <c r="B1" s="17"/>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
         <v>4</v>
       </c>
@@ -716,7 +744,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
         <v>5</v>
       </c>
@@ -724,7 +752,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
         <v>61</v>
       </c>
@@ -732,7 +760,7 @@
         <v>11228</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="12">
         <v>40.6201972</v>
       </c>
@@ -740,48 +768,61 @@
         <v>-74.015425500000006</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A7" s="16" t="s">
+    <row r="7" spans="1:3" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A7" s="18" t="s">
         <v>62</v>
       </c>
-      <c r="B7" s="17"/>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" s="14" t="s">
+      <c r="B7" s="18"/>
+      <c r="C7" s="18"/>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" s="19" t="s">
+        <v>72</v>
+      </c>
+      <c r="B8" s="14" t="s">
         <v>63</v>
       </c>
-      <c r="B8" s="15" t="s">
+      <c r="C8" s="15" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>73</v>
+      </c>
+      <c r="B9" t="s">
         <v>65</v>
       </c>
-      <c r="B9">
+      <c r="C9">
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>74</v>
+      </c>
+      <c r="B10" t="s">
         <v>66</v>
       </c>
-      <c r="B10">
+      <c r="C10">
         <v>4</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>6967</v>
+      </c>
+      <c r="B11" t="s">
         <v>67</v>
       </c>
-      <c r="B11">
+      <c r="C11">
         <v>4</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:B1"/>
-    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="A7:C7"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>